<commit_message>
docs(testing): regenerate CAA 161026 cases
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES CAA 161026.xlsx
+++ b/docs/testing/PROJECT TEST CASES CAA 161026.xlsx
@@ -7987,18 +7987,19 @@
       <c r="H145" s="2" t="inlineStr">
         <is>
           <t>1. As coord_b, submit a booking request for "Orchid Hall" for "EVT-2003 Client B Isolation Event" on 15/01/2027 13:15-15:00 (buffered window starts 12:45)
-  2. Note the outcome
-  3. Submit a second booking request for "Orchid Hall" on 15/01/2027 13:14-15:00 (buffered window starts 12:44)</t>
+2. Record the outcome; Request A must be accepted as Pending
+3. Restore this case's prepared baseline before testing Request B: remove only Request A, retain the Confirmed "EVT-101 Client A Planning Event" booking, and leave the event, Session, venue buffers and all other data as prepared
+4. From that same baseline, submit a booking request for "Orchid Hall" for "EVT-2003 Client B Isolation Event" on 15/01/2027 13:14-15:00 (buffered window starts 12:44)</t>
         </is>
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>Request A: 13:15-15:00 (buffered 12:45-15:45) | Request B: 13:14-15:00 (buffered 12:44-15:45)</t>
+          <t>Run A and B independently from the same prepared baseline: Request A: 13:15-15:00 (buffered 12:45-15:45) | Request B: 13:14-15:00 (buffered 12:44-15:45). Remove only Request A before the independent B run; retain the Confirmed EVT-101 booking.</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>Request A is accepted as Pending; Request B is blocked and the conflict names Charity Run's buffered window 09:30-12:45</t>
+          <t>From the prepared baseline, Request A is accepted as Pending. After restoring the baseline, Request B is blocked because it overlaps the Confirmed "EVT-101 Client A Planning Event" booking; the conflict names its buffered window 09:30-12:45. The original Confirmed booking remains Confirmed in both runs.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8765,7 @@
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>The event requires Wheelchair Access and a capacity of 150. For this case only, remove "Wheelchair access" from "Orchid Hall"; its seeded Theatre layout capacity is 120</t>
+          <t>The event requires the Theatre layout, Wheelchair Access and a capacity of 150. For this case only, remove "Wheelchair access" from "Orchid Hall"; its overall venue capacity is 200, but its seeded Theatre layout capacity is 120</t>
         </is>
       </c>
       <c r="H160" s="2" t="inlineStr">
@@ -8775,7 +8776,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>Event requirements: Wheelchair Access, 150 capacity | Orchid Hall: test-prepared without Wheelchair access; seeded Theatre capacity 120</t>
+          <t>Event requirements: Theatre layout, Wheelchair Access, 150 capacity | Orchid Hall: overall venue capacity 200; seeded Theatre layout capacity 120; test-prepared without Wheelchair access</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -9242,7 +9243,7 @@
       </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
-          <t>For this case only, prepare "EVT-101 Client A Planning Event" as a Confirmed event with its Event and Session period set to 15/01/2027 09:00-18:00 and a Confirmed Orchid Hall booking on 15/01/2027 10:00-12:00. Prepare "EVT-2001 Confirmed Registration Event" as a Planning event assigned to coord_b@connectsphere.com with its Event and Session period set to 15/01/2027 09:00-18:00. Orchid Hall has Turnaround time 45; coord_b@connectsphere.com is signed in as the assigned Coordinator</t>
+          <t>For this case only, prepare "EVT-101 Client A Planning Event" as a Confirmed event with its Event and Session period set to 15/01/2027 09:00-18:00 and a Confirmed Orchid Hall booking on 15/01/2027 10:00-12:00. Prepare "EVT-2001 Confirmed Registration Event" as a Planning event assigned to coord_b@connectsphere.com with its Event and Session period set to 15/01/2027 09:00-18:00. Orchid Hall has Setup time 30 and Turnaround time 45, so the existing booking's buffered window is 09:30-12:45; coord_b@connectsphere.com is signed in as the assigned Coordinator</t>
         </is>
       </c>
       <c r="H169" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(testing): regenerate corrected testcase exports
Follow-up to PR #296.
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES CAA 161026.xlsx
+++ b/docs/testing/PROJECT TEST CASES CAA 161026.xlsx
@@ -849,8 +849,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Sign-in is refused. The user remains signed out and is shown how to reset the password. A correct password does not lift the lock
-## E01-S02</t>
+          <t>Sign-in is refused. The user remains signed out and is shown how to reset the password. A correct password does not lift the lock</t>
         </is>
       </c>
     </row>
@@ -1164,8 +1163,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Activity Log contains an entry with User = organiser_a@clienta.com, Event = EVT-B01, Timestamp (to the minute), and Outcome = Access Denied
-## E01-S03</t>
+          <t>Activity Log contains an entry with User = organiser_a@clienta.com, Event = EVT-B01, Timestamp (to the minute), and Outcome = Access Denied</t>
         </is>
       </c>
     </row>
@@ -1322,8 +1320,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Only "Keynote: AI in 2027" appears in the list; "Workshop: Cloud Security" does not appear anywhere
-## E01-S04</t>
+          <t>Only "Keynote: AI in 2027" appears in the list; "Workshop: Cloud Security" does not appear anywhere</t>
         </is>
       </c>
     </row>
@@ -1584,8 +1581,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>No editable Role field/control is present; the role remains "Event Organiser" and cannot be changed from this screen
-## E01-S08</t>
+          <t>No editable Role field/control is present; the role remains "Event Organiser" and cannot be changed from this screen</t>
         </is>
       </c>
     </row>
@@ -1897,8 +1893,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>The account is not created; the Password field shows the specific policy requirement it fails (e.g. "Password must be at least 8 characters and include a number")
-## E01-S11</t>
+          <t>The account is not created; the Password field shows the specific policy requirement it fails (e.g. "Password must be at least 8 characters and include a number")</t>
         </is>
       </c>
     </row>
@@ -2159,8 +2154,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>An activity log entry exists showing actor = organiser_a@clienta.com, action = "Account Deactivated", and a timestamp
-## E01-S12</t>
+          <t>An activity log entry exists showing actor = organiser_a@clienta.com, action = "Account Deactivated", and a timestamp</t>
         </is>
       </c>
     </row>
@@ -2362,8 +2356,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>All three pass unchanged
-## E01-S13</t>
+          <t>All three pass unchanged</t>
         </is>
       </c>
     </row>
@@ -2725,8 +2718,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>All 10 named fields are present on the form and marked as mandatory
-## E02-S02</t>
+          <t>All 10 named fields are present on the form and marked as mandatory</t>
         </is>
       </c>
     </row>
@@ -2985,8 +2977,7 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>Both items are shown but visually distinguishable (e.g. a "Draft" badge on Team Offsite vs a "Submitted" status on Annual Tech Summit)
-## E02-S03</t>
+          <t>Both items are shown but visually distinguishable (e.g. a "Draft" badge on Team Offsite vs a "Submitted" status on Annual Tech Summit)</t>
         </is>
       </c>
     </row>
@@ -3142,8 +3133,7 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>Venue X is excluded from the results or clearly marked unsuitable; Venue Y appears as a normal match
-## E02-S05</t>
+          <t>Venue X is excluded from the results or clearly marked unsuitable; Venue Y appears as a normal match</t>
         </is>
       </c>
     </row>
@@ -3291,8 +3281,7 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>Submission is blocked by E02-S07 and identifies the out-of-range Session date
-## E02-S07</t>
+          <t>Submission is blocked by E02-S07 and identifies the out-of-range Session date</t>
         </is>
       </c>
     </row>
@@ -3853,8 +3842,7 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>After step 2 the assigned Coordinator is still coord_a@connectsphere.com and coord_b has been notified. After step 4 the assigned Coordinator is coord_b@connectsphere.com, the previous assignment has ended, and the change is recorded in the activity log. Each request/response notice produces one email-outbox row in the same transaction. The acting user receives no routine self-notice. Outbox failure rolls back the request or acceptance, ownership, audit and notifications
-## E03-S02</t>
+          <t>After step 2 the assigned Coordinator is still coord_a@connectsphere.com and coord_b has been notified. After step 4 the assigned Coordinator is coord_b@connectsphere.com, the previous assignment has ended, and the change is recorded in the activity log. Each request/response notice produces one email-outbox row in the same transaction. The acting user receives no routine self-notice. Outbox failure rolls back the request or acceptance, ownership, audit and notifications</t>
         </is>
       </c>
     </row>
@@ -4484,8 +4472,7 @@
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>After step 1, EVT-2003 is "Awaiting Clarification" and organiser_c@clientb.com has one notification that includes both questions. At step 2, both questions are listed with the date they were raised. After step 4, EVT-2003 is "Under Review", both questions are marked resolved with their answers linked to them, no question is outstanding, each status change is recorded in the activity log, and coord_b@connectsphere.com is notified of the response
-## E03-S03</t>
+          <t>After step 1, EVT-2003 is "Awaiting Clarification" and organiser_c@clientb.com has one notification that includes both questions. At step 2, both questions are listed with the date they were raised. After step 4, EVT-2003 is "Under Review", both questions are marked resolved with their answers linked to them, no question is outstanding, each status change is recorded in the activity log, and coord_b@connectsphere.com is notified of the response</t>
         </is>
       </c>
     </row>
@@ -5120,8 +5107,7 @@
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>Approval is not blocked: "Accessibility needs" is not listed as missing. The status becomes "Approved" and organiser_a@clienta.com is notified
-## E03-S05</t>
+          <t>Approval is not blocked: "Accessibility needs" is not listed as missing. The status becomes "Approved" and organiser_a@clienta.com is notified</t>
         </is>
       </c>
     </row>
@@ -5276,8 +5262,7 @@
       </c>
       <c r="J93" s="2" t="inlineStr">
         <is>
-          <t>All 4 past status changes are listed in order with their dates, matching the entries recorded in the activity log (E14-S02)
-## E03-S06</t>
+          <t>All 4 past status changes are listed in order with their dates, matching the entries recorded in the activity log (E14-S02)</t>
         </is>
       </c>
     </row>
@@ -5432,8 +5417,7 @@
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>The comment action is refused; organiser_b@clienta.com cannot post on an event they do not have access to
-## E03-S07</t>
+          <t>The comment action is refused; organiser_b@clienta.com cannot post on an event they do not have access to</t>
         </is>
       </c>
     </row>
@@ -5751,8 +5735,7 @@
       </c>
       <c r="J102" s="2" t="inlineStr">
         <is>
-          <t>The change is saved, and an activity log entry records the edit with actor = organiser_a@clienta.com, confirming every post-approval edit is logged regardless of who makes it
-## E03-S08</t>
+          <t>The change is saved, and an activity log entry records the edit with actor = organiser_a@clienta.com, confirming every post-approval edit is logged regardless of who makes it</t>
         </is>
       </c>
     </row>
@@ -6009,8 +5992,7 @@
       </c>
       <c r="J107" s="2" t="inlineStr">
         <is>
-          <t>The history shows Submitted at submission time and Under Review at assignment time, matching TC_E03S01_01's transition; TC_E03S05 cases continue to pass
-## E03-S09</t>
+          <t>The history shows Submitted at submission time and Under Review at assignment time, matching TC_E03S01_01's transition; TC_E03S05 cases continue to pass</t>
         </is>
       </c>
     </row>
@@ -6165,8 +6147,7 @@
       </c>
       <c r="J110" s="2" t="inlineStr">
         <is>
-          <t>The request reaches lead_1 with the reason; coordinator_1 stays assigned; after the decline coordinator_1 has a notification with the note; coordinator_2's attempt is refused as in TC_E03S01_07
-## E03-S10</t>
+          <t>The request reaches lead_1 with the reason; coordinator_1 stays assigned; after the decline coordinator_1 has a notification with the note; coordinator_2's attempt is refused as in TC_E03S01_07</t>
         </is>
       </c>
     </row>
@@ -6269,8 +6250,7 @@
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>Access is refused with no event data returned; the activity log records the denied attempt
-## E03-S12</t>
+          <t>Access is refused with no event data returned; the activity log records the denied attempt</t>
         </is>
       </c>
     </row>
@@ -7152,8 +7132,7 @@
       </c>
       <c r="J129" s="2" t="inlineStr">
         <is>
-          <t>The venue is saved with capacity 150. The booking for EVT-1001 is not flagged and no Coordinator notification is generated. Capacity equal to attendance is sufficient
-## E05-S02</t>
+          <t>The venue is saved with capacity 150. The booking for EVT-1001 is not flagged and no Coordinator notification is generated. Capacity equal to attendance is sufficient</t>
         </is>
       </c>
     </row>
@@ -7573,8 +7552,7 @@
       </c>
       <c r="J137" s="2" t="inlineStr">
         <is>
-          <t>Orchid Hall is excluded from the matching results, or shown as a near match marked unsuitable with Theatre capacity 119 below required 120 named as the failing criterion
-## E05-S03</t>
+          <t>Orchid Hall is excluded from the matching results, or shown as a near match marked unsuitable with Theatre capacity 119 below required 120 named as the failing criterion</t>
         </is>
       </c>
     </row>
@@ -7832,8 +7810,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>The entry shows Event = Annual Tech Summit, Event = the event, Date = 12/11/2026, Time = 09:00-12:00
-## E05-S04</t>
+          <t>The entry shows Event = Annual Tech Summit, Event = the event, Date = 12/11/2026, Time = 09:00-12:00</t>
         </is>
       </c>
     </row>
@@ -8051,8 +8028,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>"Riverside Hall" now appears as available from 08/01/2027 onward, while remaining blocked for 05/01/2027-07/01/2027
-## E05-S05</t>
+          <t>"Riverside Hall" now appears as available from 08/01/2027 onward, while remaining blocked for 05/01/2027-07/01/2027</t>
         </is>
       </c>
     </row>
@@ -8418,8 +8394,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>"Riverside Hall" is not offered as available for the event; where it is listed its unavailability names the 12:30-12:45 overlap with the other booking's turnaround
-## E05-S06</t>
+          <t>"Riverside Hall" is not offered as available for the event; where it is listed its unavailability names the 12:30-12:45 overlap with the other booking's turnaround</t>
         </is>
       </c>
     </row>
@@ -8941,8 +8916,7 @@
       </c>
       <c r="J163" s="2" t="inlineStr">
         <is>
-          <t>"Grand Ballroom" does not appear as available in the results for 15/11/2026
-## E06-S02</t>
+          <t>"Grand Ballroom" does not appear as available in the results for 15/11/2026</t>
         </is>
       </c>
     </row>
@@ -9210,8 +9184,7 @@
 Unsuitable and explicitly state "outside operating hours". The result is advisory,
 not a booking rejection. E06-S01 does not gain an operating-hours failure.
 Actual booking submission and Venue Staff decision display remain TC_E06S02_04
-and require the E06-S03/S04 workflows; evaluator/UI tests alone do not prove them.
-## E06-S03</t>
+and require the E06-S03/S04 workflows; evaluator/UI tests alone do not prove them.</t>
         </is>
       </c>
     </row>
@@ -9893,8 +9866,7 @@
       </c>
       <c r="J181" s="2" t="inlineStr">
         <is>
-          <t>Step 1 is refused because the Rejected B still consumes A's slot. C and D may be requested through their immediately preceding rejections, with all normal checks rerun and historical rows unchanged; there is no two-attempt maximum. No switch is offered for a rejection without a suggestion. Ordinary venue-search requests are a separate journey.
-## E06-S04</t>
+          <t>Step 1 is refused because the Rejected B still consumes A's slot. C and D may be requested through their immediately preceding rejections, with all normal checks rerun and historical rows unchanged; there is no two-attempt maximum. No switch is offered for a rejection without a suggestion. Ordinary venue-search requests are a separate journey.</t>
         </is>
       </c>
     </row>
@@ -10269,8 +10241,7 @@
       <c r="J188" s="2" t="inlineStr">
         <is>
           <t>An entry is recorded with the actor, action ("Booking Released"), the affected booking/event, and a timestamp
-Transferred from TC_E14S02_07 by T-76 on 2 October 2026.
-## E06-S05</t>
+Transferred from TC_E14S02_07 by T-76 on 2 October 2026.</t>
         </is>
       </c>
     </row>
@@ -10635,8 +10606,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>Step 1 succeeds and the activity log records the extension by venue_staff_1 with the old and new expiry; step 2 is refused with a message that an expired hold cannot be extended and must be placed again
-## E06-S06</t>
+          <t>Step 1 succeeds and the activity log records the extension by venue_staff_1 with the old and new expiry; step 2 is refused with a message that an expired hold cannot be extended and must be placed again</t>
         </is>
       </c>
     </row>
@@ -11211,8 +11181,7 @@
       </c>
       <c r="J206" s="2" t="inlineStr">
         <is>
-          <t>The updated Location value is saved and shown when the item record is reopened
-## E07-S02</t>
+          <t>The updated Location value is saved and shown when the item record is reopened</t>
         </is>
       </c>
     </row>
@@ -11426,8 +11395,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>After step 3, the request shows "Wireless Microphone x3"; after step 5, the request no longer includes "Wireless Microphone"
-## E07-S03</t>
+          <t>After step 3, the request shows "Wireless Microphone x3"; after step 5, the request no longer includes "Wireless Microphone"</t>
         </is>
       </c>
     </row>
@@ -11581,8 +11549,7 @@
       </c>
       <c r="J213" s="2" t="inlineStr">
         <is>
-          <t>"Wireless Microphone" shows its full free quantity for both the event's and the event's time windows
-## E07-S04</t>
+          <t>"Wireless Microphone" shows its full free quantity for both the event's and the event's time windows</t>
         </is>
       </c>
     </row>
@@ -11953,8 +11920,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>The reservation is recorded with status Partial. The Coordinator is notified of an outstanding quantity of 1. Confirmation is blocked and the outstanding item is listed against event EVT-1003
-## E07-S05</t>
+          <t>The reservation is recorded with status Partial. The Coordinator is notified of an outstanding quantity of 1. Confirmation is blocked and the outstanding item is listed against event EVT-1003</t>
         </is>
       </c>
     </row>
@@ -12116,8 +12082,7 @@
       </c>
       <c r="J223" s="2" t="inlineStr">
         <is>
-          <t>"HD Camera" now shows as available again for 03/12/2026
-## E07-S06</t>
+          <t>"HD Camera" now shows as available again for 03/12/2026</t>
         </is>
       </c>
     </row>
@@ -12277,8 +12242,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>No technical support request is created for the event, and later event confirmation is not blocked waiting for a staff assignment
-## E07-S07</t>
+          <t>No technical support request is created for the event, and later event confirmation is not blocked waiting for a staff assignment</t>
         </is>
       </c>
     </row>
@@ -12593,8 +12557,7 @@
       </c>
       <c r="J232" s="2" t="inlineStr">
         <is>
-          <t>tech_support_2@connectsphere.com receives a notification for the assignment, and a separate notification for the removal
-## E07-S08</t>
+          <t>tech_support_2@connectsphere.com receives a notification for the assignment, and a separate notification for the removal</t>
         </is>
       </c>
     </row>
@@ -12791,8 +12754,7 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>The assignment remains attached to the Event and does not require duplicate Session-level assignments
-## E07-S09</t>
+          <t>The assignment remains attached to the Event and does not require duplicate Session-level assignments</t>
         </is>
       </c>
     </row>
@@ -13420,8 +13382,7 @@
       </c>
       <c r="J248" s="2" t="inlineStr">
         <is>
-          <t>Step 1 is blocked and lists the Pending booking by venue; steps 2 and 3 are refused, "Charity Run" stays in Safety Review, and both attempts are in the activity log
-## E08-S04</t>
+          <t>Step 1 is blocked and lists the Pending booking by venue; steps 2 and 3 are refused, "Charity Run" stays in Safety Review, and both attempts are in the activity log</t>
         </is>
       </c>
     </row>
@@ -13734,8 +13695,7 @@
       </c>
       <c r="J254" s="2" t="inlineStr">
         <is>
-          <t>The Event moves automatically to Planning/change review, its assigned Coordinator is notified immediately, and its status is not Cancelled
-## E08-S05</t>
+          <t>The Event moves automatically to Planning/change review, its assigned Coordinator is notified immediately, and its status is not Cancelled</t>
         </is>
       </c>
     </row>
@@ -14045,8 +14005,7 @@
       </c>
       <c r="J260" s="2" t="inlineStr">
         <is>
-          <t>At 16:59:59 the status remains Confirmed. At 17:00:00 the status becomes Completed and the transition is recorded in the activity log
-## E08-S06</t>
+          <t>At 16:59:59 the status remains Confirmed. At 17:00:00 the status becomes Completed and the transition is recorded in the activity log</t>
         </is>
       </c>
     </row>
@@ -14726,8 +14685,7 @@
       </c>
       <c r="J273" s="2" t="inlineStr">
         <is>
-          <t>One active Event-level registration is created with both Sessions selected; the attendee is not registered twice
-## E09-S02</t>
+          <t>One active Event-level registration is created with both Sessions selected; the attendee is not registered twice</t>
         </is>
       </c>
     </row>
@@ -15294,8 +15252,7 @@
       </c>
       <c r="J284" s="2" t="inlineStr">
         <is>
-          <t>Combined Event capacity is 120, derived from confirmed layout capacities; it is not an independent Organiser-entered limit
-## E09-S03</t>
+          <t>Combined Event capacity is 120, derived from confirmed layout capacities; it is not an independent Organiser-entered limit</t>
         </is>
       </c>
     </row>
@@ -15761,8 +15718,7 @@
       </c>
       <c r="J293" s="2" t="inlineStr">
         <is>
-          <t>Neither Session can be registered separately before the Event window opens or after it closes; both are selectable during the Event-level window
-## E09-S04</t>
+          <t>Neither Session can be registered separately before the Event window opens or after it closes; both are selectable during the Event-level window</t>
         </is>
       </c>
     </row>
@@ -16021,8 +15977,7 @@
       </c>
       <c r="J298" s="2" t="inlineStr">
         <is>
-          <t>attendee_j@example.com is removed from the waiting list and no longer receives notifications about released places for that event
-## E09-S05</t>
+          <t>attendee_j@example.com is removed from the waiting list and no longer receives notifications about released places for that event</t>
         </is>
       </c>
     </row>
@@ -16228,8 +16183,7 @@
       </c>
       <c r="J302" s="2" t="inlineStr">
         <is>
-          <t>All three Session seats and the combined Event seat are released by one withdrawal; no partial withdrawal is recorded
-## E09-S06</t>
+          <t>All three Session seats and the combined Event seat are released by one withdrawal; no partial withdrawal is recorded</t>
         </is>
       </c>
     </row>
@@ -16437,8 +16391,7 @@
       </c>
       <c r="J306" s="2" t="inlineStr">
         <is>
-          <t>The summary shows "Registered: 5" and "Attended: 4" together, side by side
-## E09-S07</t>
+          <t>The summary shows "Registered: 5" and "Attended: 4" together, side by side</t>
         </is>
       </c>
     </row>
@@ -17008,8 +16961,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>CR-2 becomes Obsolete automatically and history records the terminal transition separately from the cancellation reason
-## E10-S02</t>
+          <t>CR-2 becomes Obsolete automatically and history records the terminal transition separately from the cancellation reason</t>
         </is>
       </c>
     </row>
@@ -17478,8 +17430,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>No Session venue booking or equipment reservation is flagged
-## E10-S03</t>
+          <t>No Session venue booking or equipment reservation is flagged</t>
         </is>
       </c>
     </row>
@@ -17675,8 +17626,7 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>The remaining Pending request becomes Obsolete and the transition is recorded in history
-## E10-S04</t>
+          <t>The remaining Pending request becomes Obsolete and the transition is recorded in history</t>
         </is>
       </c>
     </row>
@@ -17938,8 +17888,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>Both requests become Obsolete automatically and each transition is recorded; neither is labelled rejected
-## E10-S05</t>
+          <t>Both requests become Obsolete automatically and each transition is recorded; neither is labelled rejected</t>
         </is>
       </c>
     </row>
@@ -19331,8 +19280,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>The Activity log shows the status-change entry from step 3 and no "Access Denied" entry; neither "Organiser A" nor organiser_a@clienta.com appears anywhere in the log
-## E14-S03</t>
+          <t>The Activity log shows the status-change entry from step 3 and no "Access Denied" entry; neither "Organiser A" nor organiser_a@clienta.com appears anywhere in the log</t>
         </is>
       </c>
     </row>
@@ -19659,11 +19607,7 @@
       <c r="A369" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B369" s="2" t="inlineStr">
-        <is>
-          <t>Definition of Done</t>
-        </is>
-      </c>
+      <c r="B369" s="2" t="inlineStr"/>
       <c r="C369" s="2" t="inlineStr">
         <is>
           <t>Definition of Done · BDR T-51 · Week 1 §8a</t>
@@ -19711,11 +19655,7 @@
       <c r="A370" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B370" s="2" t="inlineStr">
-        <is>
-          <t>Definition of Done</t>
-        </is>
-      </c>
+      <c r="B370" s="2" t="inlineStr"/>
       <c r="C370" s="2" t="inlineStr">
         <is>
           <t>Definition of Done · BDR T-51 · Week 1 §8a</t>
@@ -19763,11 +19703,7 @@
       <c r="A371" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B371" s="2" t="inlineStr">
-        <is>
-          <t>Definition of Done</t>
-        </is>
-      </c>
+      <c r="B371" s="2" t="inlineStr"/>
       <c r="C371" s="2" t="inlineStr">
         <is>
           <t>Definition of Done · BDR T-51 · Week 1 §8a</t>

</xml_diff>